<commit_message>
Logos and August 10 Results
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\wnba\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFE4A146-5277-44DB-86C9-D1B1B7896361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B43551D-0394-4FFE-B375-54EAB25A0435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1654EDFA-4626-4D72-A032-E72CC9A130FE}"/>
   </bookViews>
@@ -16076,6 +16076,15 @@
       <c r="G486" t="s">
         <v>24</v>
       </c>
+      <c r="H486">
+        <v>95</v>
+      </c>
+      <c r="I486">
+        <v>107</v>
+      </c>
+      <c r="J486">
+        <v>0</v>
+      </c>
     </row>
     <row r="487" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A487" s="1">
@@ -16099,6 +16108,15 @@
       <c r="G487" t="s">
         <v>25</v>
       </c>
+      <c r="H487">
+        <v>107</v>
+      </c>
+      <c r="I487">
+        <v>95</v>
+      </c>
+      <c r="J487">
+        <v>0</v>
+      </c>
     </row>
     <row r="488" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A488" s="1">
@@ -16122,6 +16140,15 @@
       <c r="G488" t="s">
         <v>24</v>
       </c>
+      <c r="H488">
+        <v>88</v>
+      </c>
+      <c r="I488">
+        <v>97</v>
+      </c>
+      <c r="J488">
+        <v>0</v>
+      </c>
     </row>
     <row r="489" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A489" s="1">
@@ -16144,6 +16171,15 @@
       </c>
       <c r="G489" t="s">
         <v>25</v>
+      </c>
+      <c r="H489">
+        <v>97</v>
+      </c>
+      <c r="I489">
+        <v>88</v>
+      </c>
+      <c r="J489">
+        <v>0</v>
       </c>
     </row>
     <row r="490" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Added August 11 2026 Results
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\wnba\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B43551D-0394-4FFE-B375-54EAB25A0435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{795ED4F0-E0E0-4503-8422-AB0DB130041D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1654EDFA-4626-4D72-A032-E72CC9A130FE}"/>
   </bookViews>
@@ -16204,6 +16204,15 @@
       <c r="G490" t="s">
         <v>24</v>
       </c>
+      <c r="H490">
+        <v>92</v>
+      </c>
+      <c r="I490">
+        <v>106</v>
+      </c>
+      <c r="J490">
+        <v>0</v>
+      </c>
     </row>
     <row r="491" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A491" s="1">
@@ -16227,6 +16236,15 @@
       <c r="G491" t="s">
         <v>25</v>
       </c>
+      <c r="H491">
+        <v>106</v>
+      </c>
+      <c r="I491">
+        <v>92</v>
+      </c>
+      <c r="J491">
+        <v>0</v>
+      </c>
     </row>
     <row r="492" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A492" s="1">
@@ -16250,6 +16268,15 @@
       <c r="G492" t="s">
         <v>24</v>
       </c>
+      <c r="H492">
+        <v>94</v>
+      </c>
+      <c r="I492">
+        <v>87</v>
+      </c>
+      <c r="J492">
+        <v>0</v>
+      </c>
     </row>
     <row r="493" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A493" s="1">
@@ -16273,6 +16300,15 @@
       <c r="G493" t="s">
         <v>25</v>
       </c>
+      <c r="H493">
+        <v>87</v>
+      </c>
+      <c r="I493">
+        <v>94</v>
+      </c>
+      <c r="J493">
+        <v>0</v>
+      </c>
     </row>
     <row r="494" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A494" s="1">
@@ -16296,6 +16332,15 @@
       <c r="G494" t="s">
         <v>24</v>
       </c>
+      <c r="H494">
+        <v>76</v>
+      </c>
+      <c r="I494">
+        <v>86</v>
+      </c>
+      <c r="J494">
+        <v>0</v>
+      </c>
     </row>
     <row r="495" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A495" s="1">
@@ -16318,6 +16363,15 @@
       </c>
       <c r="G495" t="s">
         <v>25</v>
+      </c>
+      <c r="H495">
+        <v>86</v>
+      </c>
+      <c r="I495">
+        <v>76</v>
+      </c>
+      <c r="J495">
+        <v>0</v>
       </c>
     </row>
     <row r="496" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>